<commit_message>
orçamento final ae isep
</commit_message>
<xml_diff>
--- a/DRIVE/3. Operações/3.1 Projetos/26002 - SS AEISEP (Porto)/Peças escritas/ORÇAMENTO V_FINAL POR-2026-0002-SSYS.xlsx
+++ b/DRIVE/3. Operações/3.1 Projetos/26002 - SS AEISEP (Porto)/Peças escritas/ORÇAMENTO V_FINAL POR-2026-0002-SSYS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\castr\MINDSET\DRIVE\3. Operações\3.1 Projetos\26002 - SS AEISEP (Porto)\Peças escritas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA4BEF21-C347-4FEE-AF67-6AE9A6463C3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15B53B9B-3485-4DF4-BB53-42D4D9E6B9D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -629,6 +629,9 @@
     <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -661,9 +664,6 @@
     </xf>
     <xf numFmtId="4" fontId="4" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -998,11 +998,11 @@
       <c r="A2" s="35"/>
       <c r="B2" s="36"/>
       <c r="C2" s="36"/>
-      <c r="D2" s="68" t="s">
+      <c r="D2" s="57" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
       <c r="G2" s="37"/>
     </row>
     <row r="3" spans="1:7" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1112,7 +1112,7 @@
     </row>
     <row r="11" spans="1:7" ht="6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
-      <c r="B11" s="61">
+      <c r="B11" s="62">
         <v>1</v>
       </c>
       <c r="C11" s="52"/>
@@ -1123,20 +1123,20 @@
     </row>
     <row r="12" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
-      <c r="B12" s="61"/>
+      <c r="B12" s="62"/>
       <c r="C12" s="53" t="s">
         <v>16</v>
       </c>
       <c r="D12" s="54"/>
-      <c r="E12" s="66" t="s">
+      <c r="E12" s="67" t="s">
         <v>27</v>
       </c>
-      <c r="F12" s="67"/>
+      <c r="F12" s="68"/>
       <c r="G12" s="2"/>
     </row>
     <row r="13" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
-      <c r="B13" s="62"/>
+      <c r="B13" s="63"/>
       <c r="C13" s="34" t="s">
         <v>28</v>
       </c>
@@ -1147,7 +1147,7 @@
     </row>
     <row r="14" spans="1:7" ht="6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
-      <c r="B14" s="63">
+      <c r="B14" s="64">
         <v>2</v>
       </c>
       <c r="C14" s="9"/>
@@ -1158,27 +1158,27 @@
     </row>
     <row r="15" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
-      <c r="B15" s="64"/>
+      <c r="B15" s="65"/>
       <c r="C15" s="6" t="s">
         <v>17</v>
       </c>
       <c r="D15" s="7">
-        <f>101*1.3</f>
-        <v>131.30000000000001</v>
+        <f>101*1.33665</f>
+        <v>135.00164999999998</v>
       </c>
       <c r="E15" s="8">
         <f>D15*B14</f>
-        <v>262.60000000000002</v>
+        <v>270.00329999999997</v>
       </c>
       <c r="F15" s="13">
         <f>E15</f>
-        <v>262.60000000000002</v>
+        <v>270.00329999999997</v>
       </c>
       <c r="G15" s="2"/>
     </row>
     <row r="16" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
-      <c r="B16" s="65"/>
+      <c r="B16" s="66"/>
       <c r="C16" s="34" t="s">
         <v>18</v>
       </c>
@@ -1189,7 +1189,7 @@
     </row>
     <row r="17" spans="1:7" ht="6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
-      <c r="B17" s="63">
+      <c r="B17" s="64">
         <v>1</v>
       </c>
       <c r="C17" s="9"/>
@@ -1200,27 +1200,27 @@
     </row>
     <row r="18" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
-      <c r="B18" s="64"/>
+      <c r="B18" s="65"/>
       <c r="C18" s="6" t="s">
         <v>19</v>
       </c>
       <c r="D18" s="7">
-        <f>126*1.3</f>
-        <v>163.80000000000001</v>
+        <f>126*1.26985</f>
+        <v>160.00109999999998</v>
       </c>
       <c r="E18" s="8">
         <f>D18*B17</f>
-        <v>163.80000000000001</v>
+        <v>160.00109999999998</v>
       </c>
       <c r="F18" s="13">
         <f>E18</f>
-        <v>163.80000000000001</v>
+        <v>160.00109999999998</v>
       </c>
       <c r="G18" s="2"/>
     </row>
     <row r="19" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
-      <c r="B19" s="65"/>
+      <c r="B19" s="66"/>
       <c r="C19" s="34" t="s">
         <v>20</v>
       </c>
@@ -1231,7 +1231,7 @@
     </row>
     <row r="20" spans="1:7" ht="6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
-      <c r="B20" s="63">
+      <c r="B20" s="64">
         <v>4</v>
       </c>
       <c r="C20" s="9"/>
@@ -1242,27 +1242,26 @@
     </row>
     <row r="21" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
-      <c r="B21" s="64"/>
+      <c r="B21" s="65"/>
       <c r="C21" s="6" t="s">
         <v>21</v>
       </c>
       <c r="D21" s="7">
-        <f>48*1.3</f>
-        <v>62.400000000000006</v>
+        <f>48.386556*1.291655</f>
+        <v>62.498736990179999</v>
       </c>
       <c r="E21" s="8">
-        <f>B20*D21</f>
-        <v>249.60000000000002</v>
+        <v>250</v>
       </c>
       <c r="F21" s="13">
         <f>E21</f>
-        <v>249.60000000000002</v>
+        <v>250</v>
       </c>
       <c r="G21" s="2"/>
     </row>
     <row r="22" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
-      <c r="B22" s="65"/>
+      <c r="B22" s="66"/>
       <c r="C22" s="34" t="s">
         <v>22</v>
       </c>
@@ -1273,7 +1272,7 @@
     </row>
     <row r="23" spans="1:7" ht="6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
-      <c r="B23" s="63">
+      <c r="B23" s="64">
         <v>1</v>
       </c>
       <c r="C23" s="9"/>
@@ -1284,7 +1283,7 @@
     </row>
     <row r="24" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
-      <c r="B24" s="64"/>
+      <c r="B24" s="65"/>
       <c r="C24" s="56" t="s">
         <v>31</v>
       </c>
@@ -1303,7 +1302,7 @@
     </row>
     <row r="25" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
-      <c r="B25" s="65"/>
+      <c r="B25" s="66"/>
       <c r="C25" s="34" t="s">
         <v>30</v>
       </c>
@@ -1454,7 +1453,7 @@
       <c r="E58" s="44"/>
       <c r="F58" s="45">
         <f>SUM(F12,F15,F18,F24,F21)</f>
-        <v>766.00000000000011</v>
+        <v>770.00439999999992</v>
       </c>
       <c r="G58" s="46"/>
     </row>
@@ -1463,15 +1462,15 @@
       <c r="G59" s="2"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A60" s="57" t="s">
+      <c r="A60" s="58" t="s">
         <v>24</v>
       </c>
-      <c r="B60" s="58"/>
-      <c r="C60" s="58"/>
-      <c r="D60" s="58"/>
-      <c r="E60" s="58"/>
-      <c r="F60" s="58"/>
-      <c r="G60" s="59"/>
+      <c r="B60" s="59"/>
+      <c r="C60" s="59"/>
+      <c r="D60" s="59"/>
+      <c r="E60" s="59"/>
+      <c r="F60" s="59"/>
+      <c r="G60" s="60"/>
     </row>
     <row r="61" spans="1:7" ht="5.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="31"/>
@@ -1488,11 +1487,11 @@
         <v>5</v>
       </c>
       <c r="C62" s="49"/>
-      <c r="D62" s="60" t="s">
+      <c r="D62" s="61" t="s">
         <v>8</v>
       </c>
-      <c r="E62" s="60"/>
-      <c r="F62" s="60"/>
+      <c r="E62" s="61"/>
+      <c r="F62" s="61"/>
       <c r="G62" s="50"/>
     </row>
   </sheetData>

</xml_diff>